<commit_message>
Update suite aux reviews 84cfaa1ef683c8af7b41887940268a2532fb0cdb
</commit_message>
<xml_diff>
--- a/htr-FHIR/ig/StructureDefinition-fr-core-related-entity.xlsx
+++ b/htr-FHIR/ig/StructureDefinition-fr-core-related-entity.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-05-06T15:58:22+00:00</t>
+    <t>2025-05-20T10:20:09+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -394,7 +394,7 @@
     <t>Rôle joué par la personne.</t>
   </si>
   <si>
-    <t>http://hl7.org/cda/stds/core/ValueSet/CDARoleClassMutualRelationship</t>
+    <t>https://smt.esante.gouv.fr/fhir/ValueSet/jdv-role-informateur-cisis</t>
   </si>
   <si>
     <t>RelatedEntity.code</t>

</xml_diff>